<commit_message>
Add release automation and simplify report UX
</commit_message>
<xml_diff>
--- a/config/role_networks.example.xlsx
+++ b/config/role_networks.example.xlsx
@@ -1,15 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role_Networks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Role_Networks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="작성가이드" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Role_Networks'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'작성가이드'!$A$1:$B$9</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -55,9 +59,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,12 +432,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,38 +460,255 @@
           <t>서브넷마스크</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>소유부서</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>마지막 확인일</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>guest-logon</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>10.30.0.0</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>255.255.255.0</t>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>10.30.0.0/24</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>게스트 무선</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>네트워크팀</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>corp-employee</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>10.40.1.0/24</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>임직원 무선</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>네트워크팀</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>corp-employee</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>10.40.2.0/24</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>임직원 무선 추가 대역</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>네트워크팀</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>내부용</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="53" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>내용</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>필수 컬럼</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Role 이름, 네트워크 대역</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>권장 형식</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>네트워크 대역은 10.40.1.0/24 같은 CIDR 형식을 권장합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>서브넷마스크</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CIDR을 쓰지 않고 10.40.1.0처럼 네트워크 주소만 입력할 때 필요합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>여러 대역</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>같은 Role에 여러 대역이 있으면 Role 이름을 반복해서 여러 행으로 작성합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>선택 컬럼</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>설명, 소유부서, 비고, 마지막 확인일은 사내 관리용이며 보고서 매칭에는 사용하지 않습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>주의</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>CSV, HTML, 구형 .xls 파일의 확장자만 .xlsx로 바꾸면 안 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>주의</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Excel 임시 잠금 파일(~$로 시작하는 파일)은 선택하지 마세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>보안</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>이 파일을 선택하면 생성 보고서는 내부망 전용이며 실제 Role 대역이 표시됩니다.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>